<commit_message>
weekly update feb 3rd week
</commit_message>
<xml_diff>
--- a/Untitled spreadsheet.xlsx
+++ b/Untitled spreadsheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advikholalu/Desktop/insightsgraphs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848AF7E0-B51A-A54B-BEA4-29384A871892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F0D365-B697-0942-8001-1C00CE8C8FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9914" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10620" uniqueCount="1143">
   <si>
     <t>Customer Name</t>
   </si>
@@ -3299,6 +3299,174 @@
   </si>
   <si>
     <t>Chapati cravings, Better Ingredients, Nostalgic vibes</t>
+  </si>
+  <si>
+    <t>Renu b</t>
+  </si>
+  <si>
+    <t>Gopal </t>
+  </si>
+  <si>
+    <t>ravindranath bellana</t>
+  </si>
+  <si>
+    <t>Ashmi </t>
+  </si>
+  <si>
+    <t>Zeeshan alikhan</t>
+  </si>
+  <si>
+    <t>vaishnavi Vishnu zombade</t>
+  </si>
+  <si>
+    <t>Siddharth kushwaha</t>
+  </si>
+  <si>
+    <t>Mushtaq ahmad khan</t>
+  </si>
+  <si>
+    <t>Vipul kumar prem</t>
+  </si>
+  <si>
+    <t>Hinal Tailor</t>
+  </si>
+  <si>
+    <t>Palak patra</t>
+  </si>
+  <si>
+    <t>Dharmaji Jyotshna</t>
+  </si>
+  <si>
+    <t>Nikita khatri</t>
+  </si>
+  <si>
+    <t>Ashwani Kr Singh</t>
+  </si>
+  <si>
+    <t>Abid akhtar</t>
+  </si>
+  <si>
+    <t>saratha </t>
+  </si>
+  <si>
+    <t>K MANJUNATHAREDDY</t>
+  </si>
+  <si>
+    <t>shashwat Jain</t>
+  </si>
+  <si>
+    <t>V Bhagya Lakshmi</t>
+  </si>
+  <si>
+    <t>RACHIT Chauhan</t>
+  </si>
+  <si>
+    <t>Ratnesh Shukla</t>
+  </si>
+  <si>
+    <t>Supritha </t>
+  </si>
+  <si>
+    <t>kaviprasath </t>
+  </si>
+  <si>
+    <t>Shailendra kumar verma</t>
+  </si>
+  <si>
+    <t>Ratandeep Arunkumar</t>
+  </si>
+  <si>
+    <t>Monika kanagala</t>
+  </si>
+  <si>
+    <t>Tikam singh rajput</t>
+  </si>
+  <si>
+    <t>Imran khan s</t>
+  </si>
+  <si>
+    <t>Gourav kumar gurnani</t>
+  </si>
+  <si>
+    <t>Munibanaaz </t>
+  </si>
+  <si>
+    <t>Rupal Pardeshi</t>
+  </si>
+  <si>
+    <t>Akash ghildiyal</t>
+  </si>
+  <si>
+    <t>Evening snacks</t>
+  </si>
+  <si>
+    <t>Better Ingredients, Hygiene</t>
+  </si>
+  <si>
+    <t>liked it </t>
+  </si>
+  <si>
+    <t>Candy, Lollipop, Churan, Tamrind Pop, Chocolate</t>
+  </si>
+  <si>
+    <t>Mohammad Waseem Akki</t>
+  </si>
+  <si>
+    <t>Namrata manglik</t>
+  </si>
+  <si>
+    <t>Sandeesh babu</t>
+  </si>
+  <si>
+    <t>Girijesh Gupta</t>
+  </si>
+  <si>
+    <t>Namrata Angadi</t>
+  </si>
+  <si>
+    <t>saroj gupta</t>
+  </si>
+  <si>
+    <t>uttam sundesha</t>
+  </si>
+  <si>
+    <t>Hari bagavandhan</t>
+  </si>
+  <si>
+    <t>Kritika suman</t>
+  </si>
+  <si>
+    <t>Manas Ranjan Parida</t>
+  </si>
+  <si>
+    <t>Svk </t>
+  </si>
+  <si>
+    <t>While watching content(Netflix, tv, amazon prime, sports)</t>
+  </si>
+  <si>
+    <t>Diconnected in middle of the call</t>
+  </si>
+  <si>
+    <t>Amul, Haldiram's, Novelty</t>
+  </si>
+  <si>
+    <t>local shops</t>
+  </si>
+  <si>
+    <t>Nandini Sweets, Haldiram's</t>
+  </si>
+  <si>
+    <t>Prefers whatever's convenient, </t>
+  </si>
+  <si>
+    <t>Amul, </t>
+  </si>
+  <si>
+    <t>Amul, Haldiram's, Bikaji Sweets</t>
+  </si>
+  <si>
+    <t>Haldiram's, </t>
   </si>
 </sst>
 </file>
@@ -3382,7 +3550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3407,6 +3575,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -36903,22 +37072,54 @@
       <c r="Z557" s="8"/>
     </row>
     <row r="558" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A558" s="2"/>
-      <c r="B558" s="2"/>
-      <c r="C558" s="2"/>
-      <c r="D558" s="2"/>
-      <c r="E558" s="2"/>
-      <c r="F558" s="2"/>
-      <c r="G558" s="2"/>
-      <c r="H558" s="2"/>
-      <c r="I558" s="2"/>
-      <c r="J558" s="2"/>
-      <c r="K558" s="2"/>
-      <c r="L558" s="2"/>
-      <c r="M558" s="2"/>
-      <c r="N558" s="2"/>
-      <c r="O558" s="2"/>
-      <c r="P558" s="2"/>
+      <c r="A558" s="5" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B558" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C558" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D558" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E558" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F558" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G558" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H558" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I558" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J558" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K558" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L558" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M558" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N558" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O558" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P558" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q558" s="2"/>
       <c r="R558" s="2"/>
       <c r="S558" s="2"/>
@@ -36931,22 +37132,52 @@
       <c r="Z558" s="2"/>
     </row>
     <row r="559" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A559" s="2"/>
-      <c r="B559" s="2"/>
-      <c r="C559" s="2"/>
-      <c r="D559" s="2"/>
-      <c r="E559" s="2"/>
-      <c r="F559" s="2"/>
-      <c r="G559" s="2"/>
-      <c r="H559" s="2"/>
-      <c r="I559" s="2"/>
-      <c r="J559" s="2"/>
-      <c r="K559" s="2"/>
-      <c r="L559" s="2"/>
-      <c r="M559" s="2"/>
-      <c r="N559" s="2"/>
-      <c r="O559" s="2"/>
-      <c r="P559" s="2"/>
+      <c r="A559" s="5" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B559" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C559" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D559" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E559" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F559" s="6"/>
+      <c r="G559" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H559" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I559" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="J559" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K559" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L559" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M559" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N559" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O559" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P559" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q559" s="2"/>
       <c r="R559" s="2"/>
       <c r="S559" s="2"/>
@@ -36959,22 +37190,54 @@
       <c r="Z559" s="2"/>
     </row>
     <row r="560" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A560" s="2"/>
-      <c r="B560" s="2"/>
-      <c r="C560" s="2"/>
-      <c r="D560" s="2"/>
-      <c r="E560" s="2"/>
-      <c r="F560" s="2"/>
-      <c r="G560" s="2"/>
-      <c r="H560" s="2"/>
-      <c r="I560" s="2"/>
-      <c r="J560" s="2"/>
-      <c r="K560" s="2"/>
-      <c r="L560" s="2"/>
-      <c r="M560" s="2"/>
-      <c r="N560" s="2"/>
-      <c r="O560" s="2"/>
-      <c r="P560" s="2"/>
+      <c r="A560" s="5" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B560" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C560" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D560" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E560" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F560" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G560" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H560" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I560" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J560" s="5" t="s">
+        <v>1079</v>
+      </c>
+      <c r="K560" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L560" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M560" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N560" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O560" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P560" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q560" s="2"/>
       <c r="R560" s="2"/>
       <c r="S560" s="2"/>
@@ -36987,22 +37250,54 @@
       <c r="Z560" s="2"/>
     </row>
     <row r="561" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A561" s="2"/>
-      <c r="B561" s="2"/>
-      <c r="C561" s="2"/>
-      <c r="D561" s="2"/>
-      <c r="E561" s="2"/>
-      <c r="F561" s="2"/>
-      <c r="G561" s="2"/>
-      <c r="H561" s="2"/>
-      <c r="I561" s="2"/>
-      <c r="J561" s="2"/>
-      <c r="K561" s="2"/>
-      <c r="L561" s="2"/>
-      <c r="M561" s="2"/>
-      <c r="N561" s="2"/>
-      <c r="O561" s="2"/>
-      <c r="P561" s="2"/>
+      <c r="A561" s="5" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B561" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C561" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D561" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E561" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F561" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G561" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H561" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I561" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J561" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="K561" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L561" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M561" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N561" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O561" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P561" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q561" s="2"/>
       <c r="R561" s="2"/>
       <c r="S561" s="2"/>
@@ -37015,22 +37310,54 @@
       <c r="Z561" s="2"/>
     </row>
     <row r="562" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A562" s="2"/>
-      <c r="B562" s="2"/>
-      <c r="C562" s="2"/>
-      <c r="D562" s="2"/>
-      <c r="E562" s="2"/>
-      <c r="F562" s="2"/>
-      <c r="G562" s="2"/>
-      <c r="H562" s="2"/>
-      <c r="I562" s="2"/>
-      <c r="J562" s="2"/>
-      <c r="K562" s="2"/>
-      <c r="L562" s="2"/>
-      <c r="M562" s="2"/>
-      <c r="N562" s="2"/>
-      <c r="O562" s="2"/>
-      <c r="P562" s="2"/>
+      <c r="A562" s="5" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B562" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C562" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D562" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E562" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F562" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G562" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H562" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I562" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J562" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K562" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L562" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M562" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N562" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O562" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P562" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q562" s="2"/>
       <c r="R562" s="2"/>
       <c r="S562" s="2"/>
@@ -37043,22 +37370,54 @@
       <c r="Z562" s="2"/>
     </row>
     <row r="563" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A563" s="2"/>
-      <c r="B563" s="2"/>
-      <c r="C563" s="2"/>
-      <c r="D563" s="2"/>
-      <c r="E563" s="2"/>
-      <c r="F563" s="2"/>
-      <c r="G563" s="2"/>
-      <c r="H563" s="2"/>
-      <c r="I563" s="2"/>
-      <c r="J563" s="2"/>
-      <c r="K563" s="2"/>
-      <c r="L563" s="2"/>
-      <c r="M563" s="2"/>
-      <c r="N563" s="2"/>
-      <c r="O563" s="2"/>
-      <c r="P563" s="2"/>
+      <c r="A563" s="5" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B563" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C563" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D563" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E563" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F563" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G563" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H563" s="5" t="s">
+        <v>1119</v>
+      </c>
+      <c r="I563" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J563" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="K563" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L563" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M563" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N563" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O563" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P563" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q563" s="2"/>
       <c r="R563" s="2"/>
       <c r="S563" s="2"/>
@@ -37071,22 +37430,50 @@
       <c r="Z563" s="2"/>
     </row>
     <row r="564" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A564" s="2"/>
-      <c r="B564" s="2"/>
-      <c r="C564" s="2"/>
-      <c r="D564" s="2"/>
-      <c r="E564" s="2"/>
-      <c r="F564" s="2"/>
-      <c r="G564" s="2"/>
-      <c r="H564" s="2"/>
-      <c r="I564" s="2"/>
-      <c r="J564" s="2"/>
-      <c r="K564" s="2"/>
-      <c r="L564" s="2"/>
-      <c r="M564" s="2"/>
-      <c r="N564" s="2"/>
-      <c r="O564" s="2"/>
-      <c r="P564" s="2"/>
+      <c r="A564" s="5" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B564" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C564" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D564" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E564" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F564" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G564" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H564" s="6"/>
+      <c r="I564" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J564" s="6"/>
+      <c r="K564" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L564" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M564" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N564" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O564" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P564" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q564" s="2"/>
       <c r="R564" s="2"/>
       <c r="S564" s="2"/>
@@ -37099,22 +37486,52 @@
       <c r="Z564" s="2"/>
     </row>
     <row r="565" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A565" s="2"/>
-      <c r="B565" s="2"/>
-      <c r="C565" s="2"/>
-      <c r="D565" s="2"/>
-      <c r="E565" s="2"/>
-      <c r="F565" s="2"/>
-      <c r="G565" s="2"/>
-      <c r="H565" s="2"/>
-      <c r="I565" s="2"/>
-      <c r="J565" s="2"/>
-      <c r="K565" s="2"/>
-      <c r="L565" s="2"/>
-      <c r="M565" s="2"/>
-      <c r="N565" s="2"/>
-      <c r="O565" s="2"/>
-      <c r="P565" s="2"/>
+      <c r="A565" s="5" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B565" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C565" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D565" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E565" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F565" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G565" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H565" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="I565" s="6"/>
+      <c r="J565" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K565" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L565" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M565" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N565" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O565" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P565" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q565" s="2"/>
       <c r="R565" s="2"/>
       <c r="S565" s="2"/>
@@ -37127,22 +37544,54 @@
       <c r="Z565" s="2"/>
     </row>
     <row r="566" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A566" s="2"/>
-      <c r="B566" s="2"/>
-      <c r="C566" s="2"/>
-      <c r="D566" s="2"/>
-      <c r="E566" s="2"/>
-      <c r="F566" s="2"/>
-      <c r="G566" s="2"/>
-      <c r="H566" s="2"/>
-      <c r="I566" s="2"/>
-      <c r="J566" s="2"/>
-      <c r="K566" s="2"/>
-      <c r="L566" s="2"/>
-      <c r="M566" s="2"/>
-      <c r="N566" s="2"/>
-      <c r="O566" s="2"/>
-      <c r="P566" s="2"/>
+      <c r="A566" s="5" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B566" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C566" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D566" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E566" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F566" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G566" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H566" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I566" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J566" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K566" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L566" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M566" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N566" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O566" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P566" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q566" s="2"/>
       <c r="R566" s="2"/>
       <c r="S566" s="2"/>
@@ -37155,22 +37604,54 @@
       <c r="Z566" s="2"/>
     </row>
     <row r="567" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A567" s="2"/>
-      <c r="B567" s="2"/>
-      <c r="C567" s="2"/>
-      <c r="D567" s="2"/>
-      <c r="E567" s="2"/>
-      <c r="F567" s="2"/>
-      <c r="G567" s="2"/>
-      <c r="H567" s="2"/>
-      <c r="I567" s="2"/>
-      <c r="J567" s="2"/>
-      <c r="K567" s="2"/>
-      <c r="L567" s="2"/>
-      <c r="M567" s="2"/>
-      <c r="N567" s="2"/>
-      <c r="O567" s="2"/>
-      <c r="P567" s="2"/>
+      <c r="A567" s="5" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B567" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C567" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D567" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E567" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F567" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G567" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H567" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="I567" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J567" s="5" t="s">
+        <v>1120</v>
+      </c>
+      <c r="K567" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L567" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M567" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N567" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O567" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P567" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q567" s="2"/>
       <c r="R567" s="2"/>
       <c r="S567" s="2"/>
@@ -37183,22 +37664,54 @@
       <c r="Z567" s="2"/>
     </row>
     <row r="568" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A568" s="2"/>
-      <c r="B568" s="2"/>
-      <c r="C568" s="2"/>
-      <c r="D568" s="2"/>
-      <c r="E568" s="2"/>
-      <c r="F568" s="2"/>
-      <c r="G568" s="2"/>
-      <c r="H568" s="2"/>
-      <c r="I568" s="2"/>
-      <c r="J568" s="2"/>
-      <c r="K568" s="2"/>
-      <c r="L568" s="2"/>
-      <c r="M568" s="2"/>
-      <c r="N568" s="2"/>
-      <c r="O568" s="2"/>
-      <c r="P568" s="2"/>
+      <c r="A568" s="5" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B568" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C568" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D568" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E568" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F568" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G568" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H568" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I568" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J568" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K568" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L568" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M568" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N568" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O568" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P568" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q568" s="2"/>
       <c r="R568" s="2"/>
       <c r="S568" s="2"/>
@@ -37211,22 +37724,54 @@
       <c r="Z568" s="2"/>
     </row>
     <row r="569" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A569" s="2"/>
-      <c r="B569" s="2"/>
-      <c r="C569" s="2"/>
-      <c r="D569" s="2"/>
-      <c r="E569" s="2"/>
-      <c r="F569" s="2"/>
-      <c r="G569" s="2"/>
-      <c r="H569" s="2"/>
-      <c r="I569" s="2"/>
-      <c r="J569" s="2"/>
-      <c r="K569" s="2"/>
-      <c r="L569" s="2"/>
-      <c r="M569" s="2"/>
-      <c r="N569" s="2"/>
-      <c r="O569" s="2"/>
-      <c r="P569" s="2"/>
+      <c r="A569" s="5" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B569" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C569" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D569" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E569" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F569" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G569" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H569" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="I569" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J569" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K569" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L569" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M569" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N569" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O569" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P569" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q569" s="2"/>
       <c r="R569" s="2"/>
       <c r="S569" s="2"/>
@@ -37239,22 +37784,54 @@
       <c r="Z569" s="2"/>
     </row>
     <row r="570" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A570" s="2"/>
-      <c r="B570" s="2"/>
-      <c r="C570" s="2"/>
-      <c r="D570" s="2"/>
-      <c r="E570" s="2"/>
-      <c r="F570" s="2"/>
-      <c r="G570" s="2"/>
-      <c r="H570" s="2"/>
-      <c r="I570" s="2"/>
-      <c r="J570" s="2"/>
-      <c r="K570" s="2"/>
-      <c r="L570" s="2"/>
-      <c r="M570" s="2"/>
-      <c r="N570" s="2"/>
-      <c r="O570" s="2"/>
-      <c r="P570" s="2"/>
+      <c r="A570" s="5" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B570" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C570" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D570" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E570" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F570" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G570" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H570" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I570" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="J570" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="K570" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L570" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M570" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N570" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O570" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P570" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q570" s="2"/>
       <c r="R570" s="2"/>
       <c r="S570" s="2"/>
@@ -37267,22 +37844,52 @@
       <c r="Z570" s="2"/>
     </row>
     <row r="571" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A571" s="2"/>
-      <c r="B571" s="2"/>
-      <c r="C571" s="2"/>
-      <c r="D571" s="2"/>
-      <c r="E571" s="2"/>
-      <c r="F571" s="2"/>
-      <c r="G571" s="2"/>
-      <c r="H571" s="2"/>
-      <c r="I571" s="2"/>
-      <c r="J571" s="2"/>
-      <c r="K571" s="2"/>
-      <c r="L571" s="2"/>
-      <c r="M571" s="2"/>
-      <c r="N571" s="2"/>
-      <c r="O571" s="2"/>
-      <c r="P571" s="2"/>
+      <c r="A571" s="5" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B571" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C571" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D571" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E571" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F571" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G571" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H571" s="6"/>
+      <c r="I571" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J571" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K571" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L571" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M571" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N571" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O571" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P571" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q571" s="2"/>
       <c r="R571" s="2"/>
       <c r="S571" s="2"/>
@@ -37295,22 +37902,54 @@
       <c r="Z571" s="2"/>
     </row>
     <row r="572" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A572" s="2"/>
-      <c r="B572" s="2"/>
-      <c r="C572" s="2"/>
-      <c r="D572" s="2"/>
-      <c r="E572" s="2"/>
-      <c r="F572" s="2"/>
-      <c r="G572" s="2"/>
-      <c r="H572" s="2"/>
-      <c r="I572" s="2"/>
-      <c r="J572" s="2"/>
-      <c r="K572" s="2"/>
-      <c r="L572" s="2"/>
-      <c r="M572" s="2"/>
-      <c r="N572" s="2"/>
-      <c r="O572" s="2"/>
-      <c r="P572" s="2"/>
+      <c r="A572" s="5" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B572" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C572" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D572" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E572" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F572" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G572" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H572" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I572" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J572" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K572" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L572" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M572" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N572" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O572" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P572" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q572" s="2"/>
       <c r="R572" s="2"/>
       <c r="S572" s="2"/>
@@ -37323,22 +37962,54 @@
       <c r="Z572" s="2"/>
     </row>
     <row r="573" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A573" s="2"/>
-      <c r="B573" s="2"/>
-      <c r="C573" s="2"/>
-      <c r="D573" s="2"/>
-      <c r="E573" s="2"/>
-      <c r="F573" s="2"/>
-      <c r="G573" s="2"/>
-      <c r="H573" s="2"/>
-      <c r="I573" s="2"/>
-      <c r="J573" s="2"/>
-      <c r="K573" s="2"/>
-      <c r="L573" s="2"/>
-      <c r="M573" s="2"/>
-      <c r="N573" s="2"/>
-      <c r="O573" s="2"/>
-      <c r="P573" s="2"/>
+      <c r="A573" s="5" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B573" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C573" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D573" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E573" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F573" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G573" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H573" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="I573" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J573" s="5" t="s">
+        <v>1121</v>
+      </c>
+      <c r="K573" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L573" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M573" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N573" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O573" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P573" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q573" s="2"/>
       <c r="R573" s="2"/>
       <c r="S573" s="2"/>
@@ -37351,22 +38022,54 @@
       <c r="Z573" s="2"/>
     </row>
     <row r="574" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A574" s="2"/>
-      <c r="B574" s="2"/>
-      <c r="C574" s="2"/>
-      <c r="D574" s="2"/>
-      <c r="E574" s="2"/>
-      <c r="F574" s="2"/>
-      <c r="G574" s="2"/>
-      <c r="H574" s="2"/>
-      <c r="I574" s="2"/>
-      <c r="J574" s="2"/>
-      <c r="K574" s="2"/>
-      <c r="L574" s="2"/>
-      <c r="M574" s="2"/>
-      <c r="N574" s="2"/>
-      <c r="O574" s="2"/>
-      <c r="P574" s="2"/>
+      <c r="A574" s="5" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B574" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C574" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D574" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E574" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F574" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G574" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H574" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="I574" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J574" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="K574" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L574" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M574" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N574" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O574" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P574" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q574" s="2"/>
       <c r="R574" s="2"/>
       <c r="S574" s="2"/>
@@ -37379,22 +38082,50 @@
       <c r="Z574" s="2"/>
     </row>
     <row r="575" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A575" s="2"/>
-      <c r="B575" s="2"/>
-      <c r="C575" s="2"/>
-      <c r="D575" s="2"/>
-      <c r="E575" s="2"/>
-      <c r="F575" s="2"/>
-      <c r="G575" s="2"/>
-      <c r="H575" s="2"/>
-      <c r="I575" s="2"/>
-      <c r="J575" s="2"/>
-      <c r="K575" s="2"/>
-      <c r="L575" s="2"/>
-      <c r="M575" s="2"/>
-      <c r="N575" s="2"/>
-      <c r="O575" s="2"/>
-      <c r="P575" s="2"/>
+      <c r="A575" s="5" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B575" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C575" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D575" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E575" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F575" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G575" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H575" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I575" s="6"/>
+      <c r="J575" s="6"/>
+      <c r="K575" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L575" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M575" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N575" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O575" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P575" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q575" s="2"/>
       <c r="R575" s="2"/>
       <c r="S575" s="2"/>
@@ -37407,22 +38138,54 @@
       <c r="Z575" s="2"/>
     </row>
     <row r="576" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A576" s="2"/>
-      <c r="B576" s="2"/>
-      <c r="C576" s="2"/>
-      <c r="D576" s="2"/>
-      <c r="E576" s="2"/>
-      <c r="F576" s="2"/>
-      <c r="G576" s="2"/>
-      <c r="H576" s="2"/>
-      <c r="I576" s="2"/>
-      <c r="J576" s="2"/>
-      <c r="K576" s="2"/>
-      <c r="L576" s="2"/>
-      <c r="M576" s="2"/>
-      <c r="N576" s="2"/>
-      <c r="O576" s="2"/>
-      <c r="P576" s="2"/>
+      <c r="A576" s="5" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B576" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C576" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D576" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E576" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F576" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G576" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H576" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I576" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J576" s="5" t="s">
+        <v>918</v>
+      </c>
+      <c r="K576" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L576" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M576" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N576" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O576" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P576" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q576" s="2"/>
       <c r="R576" s="2"/>
       <c r="S576" s="2"/>
@@ -37435,22 +38198,54 @@
       <c r="Z576" s="2"/>
     </row>
     <row r="577" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A577" s="2"/>
-      <c r="B577" s="2"/>
-      <c r="C577" s="2"/>
-      <c r="D577" s="2"/>
-      <c r="E577" s="2"/>
-      <c r="F577" s="2"/>
-      <c r="G577" s="2"/>
-      <c r="H577" s="2"/>
-      <c r="I577" s="2"/>
-      <c r="J577" s="2"/>
-      <c r="K577" s="2"/>
-      <c r="L577" s="2"/>
-      <c r="M577" s="2"/>
-      <c r="N577" s="2"/>
-      <c r="O577" s="2"/>
-      <c r="P577" s="2"/>
+      <c r="A577" s="5" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B577" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C577" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D577" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E577" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F577" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G577" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H577" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I577" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J577" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K577" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L577" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M577" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N577" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O577" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P577" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q577" s="2"/>
       <c r="R577" s="2"/>
       <c r="S577" s="2"/>
@@ -37463,22 +38258,54 @@
       <c r="Z577" s="2"/>
     </row>
     <row r="578" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A578" s="2"/>
-      <c r="B578" s="2"/>
-      <c r="C578" s="2"/>
-      <c r="D578" s="2"/>
-      <c r="E578" s="2"/>
-      <c r="F578" s="2"/>
-      <c r="G578" s="2"/>
-      <c r="H578" s="2"/>
-      <c r="I578" s="2"/>
-      <c r="J578" s="2"/>
-      <c r="K578" s="2"/>
-      <c r="L578" s="2"/>
-      <c r="M578" s="2"/>
-      <c r="N578" s="2"/>
-      <c r="O578" s="2"/>
-      <c r="P578" s="2"/>
+      <c r="A578" s="5" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B578" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C578" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D578" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E578" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F578" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G578" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H578" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="I578" s="5" t="s">
+        <v>1122</v>
+      </c>
+      <c r="J578" s="5" t="s">
+        <v>924</v>
+      </c>
+      <c r="K578" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L578" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M578" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N578" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O578" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P578" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q578" s="2"/>
       <c r="R578" s="2"/>
       <c r="S578" s="2"/>
@@ -37491,22 +38318,54 @@
       <c r="Z578" s="2"/>
     </row>
     <row r="579" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A579" s="2"/>
-      <c r="B579" s="2"/>
-      <c r="C579" s="2"/>
-      <c r="D579" s="2"/>
-      <c r="E579" s="2"/>
-      <c r="F579" s="2"/>
-      <c r="G579" s="2"/>
-      <c r="H579" s="2"/>
-      <c r="I579" s="2"/>
-      <c r="J579" s="2"/>
-      <c r="K579" s="2"/>
-      <c r="L579" s="2"/>
-      <c r="M579" s="2"/>
-      <c r="N579" s="2"/>
-      <c r="O579" s="2"/>
-      <c r="P579" s="2"/>
+      <c r="A579" s="5" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B579" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C579" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D579" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E579" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F579" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G579" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H579" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="I579" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J579" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="K579" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L579" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M579" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N579" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O579" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P579" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q579" s="2"/>
       <c r="R579" s="2"/>
       <c r="S579" s="2"/>
@@ -37519,22 +38378,54 @@
       <c r="Z579" s="2"/>
     </row>
     <row r="580" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A580" s="2"/>
-      <c r="B580" s="2"/>
-      <c r="C580" s="2"/>
-      <c r="D580" s="2"/>
-      <c r="E580" s="2"/>
-      <c r="F580" s="2"/>
-      <c r="G580" s="2"/>
-      <c r="H580" s="2"/>
-      <c r="I580" s="2"/>
-      <c r="J580" s="2"/>
-      <c r="K580" s="2"/>
-      <c r="L580" s="2"/>
-      <c r="M580" s="2"/>
-      <c r="N580" s="2"/>
-      <c r="O580" s="2"/>
-      <c r="P580" s="2"/>
+      <c r="A580" s="5" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B580" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C580" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D580" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E580" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F580" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G580" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H580" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I580" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J580" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K580" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L580" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M580" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N580" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O580" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P580" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q580" s="2"/>
       <c r="R580" s="2"/>
       <c r="S580" s="2"/>
@@ -37547,22 +38438,54 @@
       <c r="Z580" s="2"/>
     </row>
     <row r="581" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A581" s="2"/>
-      <c r="B581" s="2"/>
-      <c r="C581" s="2"/>
-      <c r="D581" s="2"/>
-      <c r="E581" s="2"/>
-      <c r="F581" s="2"/>
-      <c r="G581" s="2"/>
-      <c r="H581" s="2"/>
-      <c r="I581" s="2"/>
-      <c r="J581" s="2"/>
-      <c r="K581" s="2"/>
-      <c r="L581" s="2"/>
-      <c r="M581" s="2"/>
-      <c r="N581" s="2"/>
-      <c r="O581" s="2"/>
-      <c r="P581" s="2"/>
+      <c r="A581" s="5" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B581" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C581" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D581" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E581" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F581" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G581" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H581" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I581" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J581" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K581" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L581" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M581" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N581" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O581" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P581" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q581" s="2"/>
       <c r="R581" s="2"/>
       <c r="S581" s="2"/>
@@ -37575,22 +38498,52 @@
       <c r="Z581" s="2"/>
     </row>
     <row r="582" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A582" s="2"/>
-      <c r="B582" s="2"/>
-      <c r="C582" s="2"/>
-      <c r="D582" s="2"/>
-      <c r="E582" s="2"/>
-      <c r="F582" s="2"/>
-      <c r="G582" s="2"/>
-      <c r="H582" s="2"/>
-      <c r="I582" s="2"/>
-      <c r="J582" s="2"/>
-      <c r="K582" s="2"/>
-      <c r="L582" s="2"/>
-      <c r="M582" s="2"/>
-      <c r="N582" s="2"/>
-      <c r="O582" s="2"/>
-      <c r="P582" s="2"/>
+      <c r="A582" s="5" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B582" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C582" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D582" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E582" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F582" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G582" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H582" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I582" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J582" s="6"/>
+      <c r="K582" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L582" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M582" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N582" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O582" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P582" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q582" s="2"/>
       <c r="R582" s="2"/>
       <c r="S582" s="2"/>
@@ -37603,22 +38556,54 @@
       <c r="Z582" s="2"/>
     </row>
     <row r="583" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A583" s="2"/>
-      <c r="B583" s="2"/>
-      <c r="C583" s="2"/>
-      <c r="D583" s="2"/>
-      <c r="E583" s="2"/>
-      <c r="F583" s="2"/>
-      <c r="G583" s="2"/>
-      <c r="H583" s="2"/>
-      <c r="I583" s="2"/>
-      <c r="J583" s="2"/>
-      <c r="K583" s="2"/>
-      <c r="L583" s="2"/>
-      <c r="M583" s="2"/>
-      <c r="N583" s="2"/>
-      <c r="O583" s="2"/>
-      <c r="P583" s="2"/>
+      <c r="A583" s="5" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B583" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C583" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D583" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E583" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F583" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G583" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H583" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I583" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J583" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K583" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L583" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M583" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N583" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O583" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P583" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q583" s="2"/>
       <c r="R583" s="2"/>
       <c r="S583" s="2"/>
@@ -37631,22 +38616,54 @@
       <c r="Z583" s="2"/>
     </row>
     <row r="584" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A584" s="2"/>
-      <c r="B584" s="2"/>
-      <c r="C584" s="2"/>
-      <c r="D584" s="2"/>
-      <c r="E584" s="2"/>
-      <c r="F584" s="2"/>
-      <c r="G584" s="2"/>
-      <c r="H584" s="2"/>
-      <c r="I584" s="2"/>
-      <c r="J584" s="2"/>
-      <c r="K584" s="2"/>
-      <c r="L584" s="2"/>
-      <c r="M584" s="2"/>
-      <c r="N584" s="2"/>
-      <c r="O584" s="2"/>
-      <c r="P584" s="2"/>
+      <c r="A584" s="5" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B584" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C584" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D584" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E584" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F584" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G584" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H584" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="I584" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J584" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K584" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L584" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M584" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N584" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O584" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P584" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q584" s="2"/>
       <c r="R584" s="2"/>
       <c r="S584" s="2"/>
@@ -37659,22 +38676,54 @@
       <c r="Z584" s="2"/>
     </row>
     <row r="585" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A585" s="2"/>
-      <c r="B585" s="2"/>
-      <c r="C585" s="2"/>
-      <c r="D585" s="2"/>
-      <c r="E585" s="2"/>
-      <c r="F585" s="2"/>
-      <c r="G585" s="2"/>
-      <c r="H585" s="2"/>
-      <c r="I585" s="2"/>
-      <c r="J585" s="2"/>
-      <c r="K585" s="2"/>
-      <c r="L585" s="2"/>
-      <c r="M585" s="2"/>
-      <c r="N585" s="2"/>
-      <c r="O585" s="2"/>
-      <c r="P585" s="2"/>
+      <c r="A585" s="5" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B585" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C585" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D585" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E585" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F585" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G585" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H585" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I585" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J585" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="K585" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L585" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M585" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N585" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O585" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P585" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q585" s="2"/>
       <c r="R585" s="2"/>
       <c r="S585" s="2"/>
@@ -37687,22 +38736,54 @@
       <c r="Z585" s="2"/>
     </row>
     <row r="586" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A586" s="2"/>
-      <c r="B586" s="2"/>
-      <c r="C586" s="2"/>
-      <c r="D586" s="2"/>
-      <c r="E586" s="2"/>
-      <c r="F586" s="2"/>
-      <c r="G586" s="2"/>
-      <c r="H586" s="2"/>
-      <c r="I586" s="2"/>
-      <c r="J586" s="2"/>
-      <c r="K586" s="2"/>
-      <c r="L586" s="2"/>
-      <c r="M586" s="2"/>
-      <c r="N586" s="2"/>
-      <c r="O586" s="2"/>
-      <c r="P586" s="2"/>
+      <c r="A586" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="B586" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C586" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D586" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E586" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F586" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G586" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H586" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I586" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="J586" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K586" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L586" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M586" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N586" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O586" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P586" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q586" s="2"/>
       <c r="R586" s="2"/>
       <c r="S586" s="2"/>
@@ -37715,22 +38796,54 @@
       <c r="Z586" s="2"/>
     </row>
     <row r="587" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A587" s="2"/>
-      <c r="B587" s="2"/>
-      <c r="C587" s="2"/>
-      <c r="D587" s="2"/>
-      <c r="E587" s="2"/>
-      <c r="F587" s="2"/>
-      <c r="G587" s="2"/>
-      <c r="H587" s="2"/>
-      <c r="I587" s="2"/>
-      <c r="J587" s="2"/>
-      <c r="K587" s="2"/>
-      <c r="L587" s="2"/>
-      <c r="M587" s="2"/>
-      <c r="N587" s="2"/>
-      <c r="O587" s="2"/>
-      <c r="P587" s="2"/>
+      <c r="A587" s="5" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B587" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C587" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D587" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E587" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F587" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G587" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H587" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I587" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="J587" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="K587" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L587" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M587" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N587" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O587" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P587" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q587" s="2"/>
       <c r="R587" s="2"/>
       <c r="S587" s="2"/>
@@ -37743,22 +38856,54 @@
       <c r="Z587" s="2"/>
     </row>
     <row r="588" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A588" s="2"/>
-      <c r="B588" s="2"/>
-      <c r="C588" s="2"/>
-      <c r="D588" s="2"/>
-      <c r="E588" s="2"/>
-      <c r="F588" s="2"/>
-      <c r="G588" s="2"/>
-      <c r="H588" s="2"/>
-      <c r="I588" s="2"/>
-      <c r="J588" s="2"/>
-      <c r="K588" s="2"/>
-      <c r="L588" s="2"/>
-      <c r="M588" s="2"/>
-      <c r="N588" s="2"/>
-      <c r="O588" s="2"/>
-      <c r="P588" s="2"/>
+      <c r="A588" s="5" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B588" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C588" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D588" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E588" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F588" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G588" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H588" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="I588" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J588" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="K588" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L588" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M588" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N588" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O588" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P588" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q588" s="2"/>
       <c r="R588" s="2"/>
       <c r="S588" s="2"/>
@@ -37771,22 +38916,54 @@
       <c r="Z588" s="2"/>
     </row>
     <row r="589" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A589" s="2"/>
-      <c r="B589" s="2"/>
-      <c r="C589" s="2"/>
-      <c r="D589" s="2"/>
-      <c r="E589" s="2"/>
-      <c r="F589" s="2"/>
-      <c r="G589" s="2"/>
-      <c r="H589" s="2"/>
-      <c r="I589" s="2"/>
-      <c r="J589" s="2"/>
-      <c r="K589" s="2"/>
-      <c r="L589" s="2"/>
-      <c r="M589" s="2"/>
-      <c r="N589" s="2"/>
-      <c r="O589" s="2"/>
-      <c r="P589" s="2"/>
+      <c r="A589" s="5" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B589" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C589" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D589" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E589" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F589" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G589" s="5" t="s">
+        <v>896</v>
+      </c>
+      <c r="H589" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="I589" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J589" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="K589" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L589" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M589" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N589" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O589" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P589" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="Q589" s="2"/>
       <c r="R589" s="2"/>
       <c r="S589" s="2"/>
@@ -37798,51 +38975,113 @@
       <c r="Y589" s="2"/>
       <c r="Z589" s="2"/>
     </row>
-    <row r="590" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A590" s="2"/>
-      <c r="B590" s="2"/>
-      <c r="C590" s="2"/>
-      <c r="D590" s="2"/>
-      <c r="E590" s="2"/>
-      <c r="F590" s="2"/>
-      <c r="G590" s="2"/>
-      <c r="H590" s="2"/>
-      <c r="I590" s="2"/>
-      <c r="J590" s="2"/>
-      <c r="K590" s="2"/>
-      <c r="L590" s="2"/>
-      <c r="M590" s="2"/>
-      <c r="N590" s="2"/>
-      <c r="O590" s="2"/>
-      <c r="P590" s="2"/>
-      <c r="Q590" s="2"/>
-      <c r="R590" s="2"/>
-      <c r="S590" s="2"/>
-      <c r="T590" s="2"/>
-      <c r="U590" s="2"/>
-      <c r="V590" s="2"/>
-      <c r="W590" s="2"/>
-      <c r="X590" s="2"/>
-      <c r="Y590" s="2"/>
-      <c r="Z590" s="2"/>
+    <row r="590" spans="1:26" s="12" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+      <c r="A590" s="10" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B590" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C590" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D590" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E590" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F590" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G590" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H590" s="10" t="s">
+        <v>909</v>
+      </c>
+      <c r="I590" s="14"/>
+      <c r="J590" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="K590" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="L590" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M590" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N590" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="O590" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="P590" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q590" s="8"/>
+      <c r="R590" s="8"/>
+      <c r="S590" s="8"/>
+      <c r="T590" s="8"/>
+      <c r="U590" s="8"/>
+      <c r="V590" s="8"/>
+      <c r="W590" s="8"/>
+      <c r="X590" s="8"/>
+      <c r="Y590" s="8"/>
+      <c r="Z590" s="8"/>
     </row>
     <row r="591" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A591" s="2"/>
-      <c r="B591" s="2"/>
-      <c r="C591" s="2"/>
-      <c r="D591" s="2"/>
-      <c r="E591" s="2"/>
-      <c r="F591" s="2"/>
-      <c r="G591" s="2"/>
-      <c r="H591" s="2"/>
-      <c r="I591" s="2"/>
-      <c r="J591" s="2"/>
-      <c r="K591" s="2"/>
-      <c r="L591" s="2"/>
-      <c r="M591" s="2"/>
-      <c r="N591" s="2"/>
-      <c r="O591" s="2"/>
-      <c r="P591" s="2"/>
+      <c r="A591" s="5" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B591" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C591" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D591" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E591" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F591" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G591" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H591" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I591" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J591" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K591" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L591" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="M591" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="N591" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="O591" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P591" s="5" t="s">
+        <v>262</v>
+      </c>
       <c r="Q591" s="2"/>
       <c r="R591" s="2"/>
       <c r="S591" s="2"/>
@@ -37855,22 +39094,54 @@
       <c r="Z591" s="2"/>
     </row>
     <row r="592" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A592" s="2"/>
-      <c r="B592" s="2"/>
-      <c r="C592" s="2"/>
-      <c r="D592" s="2"/>
-      <c r="E592" s="2"/>
-      <c r="F592" s="2"/>
-      <c r="G592" s="2"/>
-      <c r="H592" s="2"/>
-      <c r="I592" s="2"/>
-      <c r="J592" s="2"/>
-      <c r="K592" s="2"/>
-      <c r="L592" s="2"/>
-      <c r="M592" s="2"/>
-      <c r="N592" s="2"/>
-      <c r="O592" s="2"/>
-      <c r="P592" s="2"/>
+      <c r="A592" s="5" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B592" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C592" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D592" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E592" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F592" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G592" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H592" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I592" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J592" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K592" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L592" s="5" t="s">
+        <v>1135</v>
+      </c>
+      <c r="M592" s="5" t="s">
+        <v>1135</v>
+      </c>
+      <c r="N592" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="O592" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="P592" s="5" t="s">
+        <v>260</v>
+      </c>
       <c r="Q592" s="2"/>
       <c r="R592" s="2"/>
       <c r="S592" s="2"/>
@@ -37883,22 +39154,54 @@
       <c r="Z592" s="2"/>
     </row>
     <row r="593" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A593" s="2"/>
-      <c r="B593" s="2"/>
-      <c r="C593" s="2"/>
-      <c r="D593" s="2"/>
-      <c r="E593" s="2"/>
-      <c r="F593" s="2"/>
-      <c r="G593" s="2"/>
-      <c r="H593" s="2"/>
-      <c r="I593" s="2"/>
-      <c r="J593" s="2"/>
-      <c r="K593" s="2"/>
-      <c r="L593" s="2"/>
-      <c r="M593" s="2"/>
-      <c r="N593" s="2"/>
-      <c r="O593" s="2"/>
-      <c r="P593" s="2"/>
+      <c r="A593" s="5" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B593" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C593" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D593" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E593" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F593" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G593" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H593" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I593" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J593" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K593" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L593" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="M593" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="N593" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="O593" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="P593" s="5" t="s">
+        <v>267</v>
+      </c>
       <c r="Q593" s="2"/>
       <c r="R593" s="2"/>
       <c r="S593" s="2"/>
@@ -37911,22 +39214,54 @@
       <c r="Z593" s="2"/>
     </row>
     <row r="594" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A594" s="2"/>
-      <c r="B594" s="2"/>
-      <c r="C594" s="2"/>
-      <c r="D594" s="2"/>
-      <c r="E594" s="2"/>
-      <c r="F594" s="2"/>
-      <c r="G594" s="2"/>
-      <c r="H594" s="2"/>
-      <c r="I594" s="2"/>
-      <c r="J594" s="2"/>
-      <c r="K594" s="2"/>
-      <c r="L594" s="2"/>
-      <c r="M594" s="2"/>
-      <c r="N594" s="2"/>
-      <c r="O594" s="2"/>
-      <c r="P594" s="2"/>
+      <c r="A594" s="5" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B594" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C594" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D594" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E594" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F594" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G594" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H594" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I594" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J594" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K594" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L594" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="M594" s="5" t="s">
+        <v>1136</v>
+      </c>
+      <c r="N594" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="O594" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="P594" s="5" t="s">
+        <v>260</v>
+      </c>
       <c r="Q594" s="2"/>
       <c r="R594" s="2"/>
       <c r="S594" s="2"/>
@@ -37939,22 +39274,54 @@
       <c r="Z594" s="2"/>
     </row>
     <row r="595" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A595" s="2"/>
-      <c r="B595" s="2"/>
-      <c r="C595" s="2"/>
-      <c r="D595" s="2"/>
-      <c r="E595" s="2"/>
-      <c r="F595" s="2"/>
-      <c r="G595" s="2"/>
-      <c r="H595" s="2"/>
-      <c r="I595" s="2"/>
-      <c r="J595" s="2"/>
-      <c r="K595" s="2"/>
-      <c r="L595" s="2"/>
-      <c r="M595" s="2"/>
-      <c r="N595" s="2"/>
-      <c r="O595" s="2"/>
-      <c r="P595" s="2"/>
+      <c r="A595" s="5" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B595" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C595" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D595" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E595" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F595" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G595" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H595" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I595" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J595" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K595" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L595" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="M595" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="N595" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="O595" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P595" s="5" t="s">
+        <v>319</v>
+      </c>
       <c r="Q595" s="2"/>
       <c r="R595" s="2"/>
       <c r="S595" s="2"/>
@@ -37967,22 +39334,52 @@
       <c r="Z595" s="2"/>
     </row>
     <row r="596" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A596" s="2"/>
-      <c r="B596" s="2"/>
-      <c r="C596" s="2"/>
-      <c r="D596" s="2"/>
-      <c r="E596" s="2"/>
-      <c r="F596" s="2"/>
-      <c r="G596" s="2"/>
-      <c r="H596" s="2"/>
-      <c r="I596" s="2"/>
-      <c r="J596" s="2"/>
-      <c r="K596" s="2"/>
-      <c r="L596" s="2"/>
-      <c r="M596" s="2"/>
-      <c r="N596" s="2"/>
-      <c r="O596" s="2"/>
-      <c r="P596" s="2"/>
+      <c r="A596" s="5" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B596" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C596" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D596" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E596" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F596" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G596" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H596" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I596" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J596" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K596" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L596" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="M596" s="5" t="s">
+        <v>1137</v>
+      </c>
+      <c r="N596" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="O596" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P596" s="6"/>
       <c r="Q596" s="2"/>
       <c r="R596" s="2"/>
       <c r="S596" s="2"/>
@@ -37995,22 +39392,52 @@
       <c r="Z596" s="2"/>
     </row>
     <row r="597" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A597" s="2"/>
-      <c r="B597" s="2"/>
-      <c r="C597" s="2"/>
-      <c r="D597" s="2"/>
-      <c r="E597" s="2"/>
-      <c r="F597" s="2"/>
-      <c r="G597" s="2"/>
-      <c r="H597" s="2"/>
-      <c r="I597" s="2"/>
-      <c r="J597" s="2"/>
-      <c r="K597" s="2"/>
-      <c r="L597" s="2"/>
-      <c r="M597" s="2"/>
-      <c r="N597" s="2"/>
-      <c r="O597" s="2"/>
-      <c r="P597" s="2"/>
+      <c r="A597" s="5" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B597" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C597" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D597" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E597" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F597" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G597" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H597" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I597" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J597" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K597" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L597" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="M597" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="N597" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="O597" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P597" s="6"/>
       <c r="Q597" s="2"/>
       <c r="R597" s="2"/>
       <c r="S597" s="2"/>
@@ -38023,22 +39450,54 @@
       <c r="Z597" s="2"/>
     </row>
     <row r="598" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A598" s="2"/>
-      <c r="B598" s="2"/>
-      <c r="C598" s="2"/>
-      <c r="D598" s="2"/>
-      <c r="E598" s="2"/>
-      <c r="F598" s="2"/>
-      <c r="G598" s="2"/>
-      <c r="H598" s="2"/>
-      <c r="I598" s="2"/>
-      <c r="J598" s="2"/>
-      <c r="K598" s="2"/>
-      <c r="L598" s="2"/>
-      <c r="M598" s="2"/>
-      <c r="N598" s="2"/>
-      <c r="O598" s="2"/>
-      <c r="P598" s="2"/>
+      <c r="A598" s="5" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B598" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C598" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D598" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E598" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F598" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G598" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H598" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I598" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J598" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K598" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L598" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="M598" s="5" t="s">
+        <v>1138</v>
+      </c>
+      <c r="N598" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="O598" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="P598" s="5" t="s">
+        <v>1134</v>
+      </c>
       <c r="Q598" s="2"/>
       <c r="R598" s="2"/>
       <c r="S598" s="2"/>
@@ -38051,22 +39510,52 @@
       <c r="Z598" s="2"/>
     </row>
     <row r="599" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A599" s="2"/>
-      <c r="B599" s="2"/>
-      <c r="C599" s="2"/>
-      <c r="D599" s="2"/>
-      <c r="E599" s="2"/>
-      <c r="F599" s="2"/>
-      <c r="G599" s="2"/>
-      <c r="H599" s="2"/>
-      <c r="I599" s="2"/>
-      <c r="J599" s="2"/>
-      <c r="K599" s="2"/>
-      <c r="L599" s="2"/>
-      <c r="M599" s="2"/>
-      <c r="N599" s="2"/>
-      <c r="O599" s="2"/>
-      <c r="P599" s="2"/>
+      <c r="A599" s="5" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B599" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C599" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D599" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E599" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F599" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G599" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H599" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I599" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J599" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K599" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L599" s="6"/>
+      <c r="M599" s="5" t="s">
+        <v>1139</v>
+      </c>
+      <c r="N599" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="O599" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P599" s="5" t="s">
+        <v>260</v>
+      </c>
       <c r="Q599" s="2"/>
       <c r="R599" s="2"/>
       <c r="S599" s="2"/>
@@ -38079,22 +39568,54 @@
       <c r="Z599" s="2"/>
     </row>
     <row r="600" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A600" s="2"/>
-      <c r="B600" s="2"/>
-      <c r="C600" s="2"/>
-      <c r="D600" s="2"/>
-      <c r="E600" s="2"/>
-      <c r="F600" s="2"/>
-      <c r="G600" s="2"/>
-      <c r="H600" s="2"/>
-      <c r="I600" s="2"/>
-      <c r="J600" s="2"/>
-      <c r="K600" s="2"/>
-      <c r="L600" s="2"/>
-      <c r="M600" s="2"/>
-      <c r="N600" s="2"/>
-      <c r="O600" s="2"/>
-      <c r="P600" s="2"/>
+      <c r="A600" s="5" t="s">
+        <v>944</v>
+      </c>
+      <c r="B600" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C600" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D600" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E600" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F600" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G600" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H600" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I600" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J600" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K600" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L600" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="M600" s="5" t="s">
+        <v>1140</v>
+      </c>
+      <c r="N600" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="O600" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P600" s="5" t="s">
+        <v>262</v>
+      </c>
       <c r="Q600" s="2"/>
       <c r="R600" s="2"/>
       <c r="S600" s="2"/>
@@ -38107,22 +39628,52 @@
       <c r="Z600" s="2"/>
     </row>
     <row r="601" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A601" s="2"/>
-      <c r="B601" s="2"/>
-      <c r="C601" s="2"/>
-      <c r="D601" s="2"/>
-      <c r="E601" s="2"/>
-      <c r="F601" s="2"/>
-      <c r="G601" s="2"/>
-      <c r="H601" s="2"/>
-      <c r="I601" s="2"/>
-      <c r="J601" s="2"/>
-      <c r="K601" s="2"/>
-      <c r="L601" s="2"/>
-      <c r="M601" s="2"/>
-      <c r="N601" s="2"/>
-      <c r="O601" s="2"/>
-      <c r="P601" s="2"/>
+      <c r="A601" s="5" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B601" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C601" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D601" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E601" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F601" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G601" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H601" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I601" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J601" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K601" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L601" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="M601" s="5" t="s">
+        <v>1141</v>
+      </c>
+      <c r="N601" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="O601" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="P601" s="6"/>
       <c r="Q601" s="2"/>
       <c r="R601" s="2"/>
       <c r="S601" s="2"/>
@@ -38134,33 +39685,62 @@
       <c r="Y601" s="2"/>
       <c r="Z601" s="2"/>
     </row>
-    <row r="602" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A602" s="2"/>
-      <c r="B602" s="2"/>
-      <c r="C602" s="2"/>
-      <c r="D602" s="2"/>
-      <c r="E602" s="2"/>
-      <c r="F602" s="2"/>
-      <c r="G602" s="2"/>
-      <c r="H602" s="2"/>
-      <c r="I602" s="2"/>
-      <c r="J602" s="2"/>
-      <c r="K602" s="2"/>
-      <c r="L602" s="2"/>
-      <c r="M602" s="2"/>
-      <c r="N602" s="2"/>
-      <c r="O602" s="2"/>
-      <c r="P602" s="2"/>
-      <c r="Q602" s="2"/>
-      <c r="R602" s="2"/>
-      <c r="S602" s="2"/>
-      <c r="T602" s="2"/>
-      <c r="U602" s="2"/>
-      <c r="V602" s="2"/>
-      <c r="W602" s="2"/>
-      <c r="X602" s="2"/>
-      <c r="Y602" s="2"/>
-      <c r="Z602" s="2"/>
+    <row r="602" spans="1:26" s="12" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+      <c r="A602" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B602" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C602" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D602" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="E602" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F602" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G602" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H602" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="I602" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J602" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K602" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L602" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="M602" s="10" t="s">
+        <v>1142</v>
+      </c>
+      <c r="N602" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="O602" s="10" t="s">
+        <v>896</v>
+      </c>
+      <c r="Q602" s="8"/>
+      <c r="R602" s="8"/>
+      <c r="S602" s="8"/>
+      <c r="T602" s="8"/>
+      <c r="U602" s="8"/>
+      <c r="V602" s="8"/>
+      <c r="W602" s="8"/>
+      <c r="X602" s="8"/>
+      <c r="Y602" s="8"/>
+      <c r="Z602" s="8"/>
     </row>
     <row r="603" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A603" s="2"/>

</xml_diff>

<commit_message>
Updated consumer insights tabs (filters + respondents + fixes)
</commit_message>
<xml_diff>
--- a/Untitled spreadsheet.xlsx
+++ b/Untitled spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advikholalu/Desktop/insightsgraphs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F0D365-B697-0942-8001-1C00CE8C8FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3FEDC3-7946-CA40-88E0-D258C2E7F907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Sweets" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Master!$A$1:$P$486</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Master!$A$1:$P$602</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10620" uniqueCount="1143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10622" uniqueCount="1143">
   <si>
     <t>Customer Name</t>
   </si>
@@ -28752,7 +28752,9 @@
       <c r="B418" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C418" s="6"/>
+      <c r="C418" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="D418" s="5" t="s">
         <v>97</v>
       </c>
@@ -29348,7 +29350,9 @@
       <c r="B428" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C428" s="6"/>
+      <c r="C428" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="D428" s="5" t="s">
         <v>237</v>
       </c>
@@ -50803,7 +50807,7 @@
       <c r="Z997" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P486" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P602" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>